<commit_message>
Add melt-fraction predictor (melt-only majors -> cumulative F, all melts, RMSE~0.11); refresh calibration data + meter_rank for the 58-melt scope filter (calib 1.06)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/meter_rank.xlsx
+++ b/meter_rank.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,52 +429,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Pairs</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Hygrometer train rmse</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Hygrometer test rmse</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Thermometer train rmse</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Thermometer test rmse</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Barometer train rmse</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Barometer test rmse</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>N&gt;200</t>
         </is>
@@ -586,25 +598,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1020</v>
+        <v>1006</v>
       </c>
       <c r="D5" t="n">
-        <v>0.54</v>
+        <v>0.539</v>
       </c>
       <c r="E5" t="n">
-        <v>1.043</v>
+        <v>1.063</v>
       </c>
       <c r="F5" t="n">
-        <v>10.82</v>
+        <v>10.35</v>
       </c>
       <c r="G5" t="n">
-        <v>23.81</v>
+        <v>23.55</v>
       </c>
       <c r="H5" t="n">
-        <v>0.657</v>
+        <v>0.592</v>
       </c>
       <c r="I5" t="n">
-        <v>1.772</v>
+        <v>1.775</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -726,29 +738,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>melt_only-pyxspplgsat</t>
+          <t>melt-opx</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1226</v>
+        <v>284</v>
       </c>
       <c r="D9" t="n">
-        <v>0.636</v>
+        <v>0.485</v>
       </c>
       <c r="E9" t="n">
-        <v>1.241</v>
+        <v>1.254</v>
       </c>
       <c r="F9" t="n">
-        <v>13.75</v>
+        <v>7.05</v>
       </c>
       <c r="G9" t="n">
-        <v>32.7</v>
+        <v>28.28</v>
       </c>
       <c r="H9" t="n">
-        <v>0.833</v>
+        <v>0.274</v>
       </c>
       <c r="I9" t="n">
-        <v>2.092</v>
+        <v>1.347</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -762,29 +774,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>melt-opx</t>
+          <t>melt_only-pyxspplgsat</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>284</v>
+        <v>1193</v>
       </c>
       <c r="D10" t="n">
-        <v>0.485</v>
+        <v>0.643</v>
       </c>
       <c r="E10" t="n">
-        <v>1.254</v>
+        <v>1.305</v>
       </c>
       <c r="F10" t="n">
-        <v>7.05</v>
+        <v>13.21</v>
       </c>
       <c r="G10" t="n">
-        <v>28.28</v>
+        <v>32.26</v>
       </c>
       <c r="H10" t="n">
-        <v>0.274</v>
+        <v>0.633</v>
       </c>
       <c r="I10" t="n">
-        <v>1.347</v>
+        <v>1.981</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -802,25 +814,25 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2256</v>
+        <v>2199</v>
       </c>
       <c r="D11" t="n">
-        <v>0.611</v>
+        <v>0.619</v>
       </c>
       <c r="E11" t="n">
-        <v>1.362</v>
+        <v>1.357</v>
       </c>
       <c r="F11" t="n">
-        <v>14.83</v>
+        <v>14.49</v>
       </c>
       <c r="G11" t="n">
-        <v>35.58</v>
+        <v>33.4</v>
       </c>
       <c r="H11" t="n">
-        <v>0.911</v>
+        <v>0.822</v>
       </c>
       <c r="I11" t="n">
-        <v>2.46</v>
+        <v>2.204</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update deployed model + tables to the sanity-checked database (2026-06-30): corrected calibration workbook (57 pair sheets + meltfrac), method_comparison + meter_rank rebuilt — deployed Melt_only-PlgSat hygrometer 1.06->1.00 wt%. Consistent with Part I/II.
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/meter_rank.xlsx
+++ b/meter_rank.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -486,29 +486,29 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>melt-plg</t>
+          <t>ol-plg</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>775</v>
+        <v>497</v>
       </c>
       <c r="D2" t="n">
         <v>0.28</v>
       </c>
       <c r="E2" t="n">
-        <v>0.864</v>
+        <v>0.865</v>
       </c>
       <c r="F2" t="n">
-        <v>5.27</v>
+        <v>6.78</v>
       </c>
       <c r="G2" t="n">
-        <v>18.99</v>
+        <v>26.43</v>
       </c>
       <c r="H2" t="n">
-        <v>0.309</v>
+        <v>0.499</v>
       </c>
       <c r="I2" t="n">
-        <v>1.191</v>
+        <v>1.524</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -522,29 +522,29 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ol-plg</t>
+          <t>melt-plg</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>497</v>
+        <v>775</v>
       </c>
       <c r="D3" t="n">
         <v>0.28</v>
       </c>
       <c r="E3" t="n">
-        <v>0.865</v>
+        <v>0.868</v>
       </c>
       <c r="F3" t="n">
-        <v>6.78</v>
+        <v>5.3</v>
       </c>
       <c r="G3" t="n">
-        <v>26.43</v>
+        <v>19.04</v>
       </c>
       <c r="H3" t="n">
-        <v>0.499</v>
+        <v>0.391</v>
       </c>
       <c r="I3" t="n">
-        <v>1.524</v>
+        <v>1.205</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -565,22 +565,22 @@
         <v>765</v>
       </c>
       <c r="D4" t="n">
-        <v>0.287</v>
+        <v>0.289</v>
       </c>
       <c r="E4" t="n">
-        <v>0.948</v>
+        <v>0.945</v>
       </c>
       <c r="F4" t="n">
-        <v>7.76</v>
+        <v>7.78</v>
       </c>
       <c r="G4" t="n">
-        <v>25.71</v>
+        <v>25.51</v>
       </c>
       <c r="H4" t="n">
-        <v>0.437</v>
+        <v>0.445</v>
       </c>
       <c r="I4" t="n">
-        <v>1.538</v>
+        <v>1.537</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -598,25 +598,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1006</v>
+        <v>984</v>
       </c>
       <c r="D5" t="n">
-        <v>0.539</v>
+        <v>0.533</v>
       </c>
       <c r="E5" t="n">
-        <v>1.063</v>
+        <v>0.997</v>
       </c>
       <c r="F5" t="n">
-        <v>10.35</v>
+        <v>10.97</v>
       </c>
       <c r="G5" t="n">
-        <v>23.55</v>
+        <v>24.29</v>
       </c>
       <c r="H5" t="n">
-        <v>0.592</v>
+        <v>0.641</v>
       </c>
       <c r="I5" t="n">
-        <v>1.775</v>
+        <v>1.76</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -673,22 +673,22 @@
         <v>751</v>
       </c>
       <c r="D7" t="n">
-        <v>0.375</v>
+        <v>0.38</v>
       </c>
       <c r="E7" t="n">
-        <v>1.17</v>
+        <v>1.168</v>
       </c>
       <c r="F7" t="n">
-        <v>6.7</v>
+        <v>6.72</v>
       </c>
       <c r="G7" t="n">
-        <v>26.9</v>
+        <v>26.84</v>
       </c>
       <c r="H7" t="n">
-        <v>0.178</v>
+        <v>0.177</v>
       </c>
       <c r="I7" t="n">
-        <v>1.219</v>
+        <v>1.213</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -748,19 +748,19 @@
         <v>0.485</v>
       </c>
       <c r="E9" t="n">
-        <v>1.254</v>
+        <v>1.252</v>
       </c>
       <c r="F9" t="n">
         <v>7.05</v>
       </c>
       <c r="G9" t="n">
-        <v>28.28</v>
+        <v>28.23</v>
       </c>
       <c r="H9" t="n">
-        <v>0.274</v>
+        <v>0.272</v>
       </c>
       <c r="I9" t="n">
-        <v>1.347</v>
+        <v>1.341</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -778,25 +778,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1193</v>
+        <v>1171</v>
       </c>
       <c r="D10" t="n">
-        <v>0.643</v>
+        <v>0.641</v>
       </c>
       <c r="E10" t="n">
-        <v>1.305</v>
+        <v>1.253</v>
       </c>
       <c r="F10" t="n">
-        <v>13.21</v>
+        <v>13.43</v>
       </c>
       <c r="G10" t="n">
-        <v>32.26</v>
+        <v>32.24</v>
       </c>
       <c r="H10" t="n">
-        <v>0.633</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="I10" t="n">
-        <v>1.981</v>
+        <v>1.979</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -814,25 +814,25 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2199</v>
+        <v>2173</v>
       </c>
       <c r="D11" t="n">
-        <v>0.619</v>
+        <v>0.613</v>
       </c>
       <c r="E11" t="n">
-        <v>1.357</v>
+        <v>1.33</v>
       </c>
       <c r="F11" t="n">
-        <v>14.49</v>
+        <v>14.61</v>
       </c>
       <c r="G11" t="n">
-        <v>33.4</v>
+        <v>33.99</v>
       </c>
       <c r="H11" t="n">
-        <v>0.822</v>
+        <v>0.827</v>
       </c>
       <c r="I11" t="n">
-        <v>2.204</v>
+        <v>2.242</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>

</xml_diff>